<commit_message>
WiFi Kitesurf + Paddle : nouvelle box Livebox-5B80 (02/09/2026)
Remplace BBOX - 4929C743 pour les 2 apparts uniquement (Surf et Hamac inchangés).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recap-apparts.xlsx
+++ b/recap-apparts.xlsx
@@ -3004,12 +3004,12 @@
       </c>
       <c r="AH2" s="7" t="inlineStr">
         <is>
-          <t>BBOX - 4929C743</t>
+          <t>Livebox-5B80</t>
         </is>
       </c>
       <c r="AI2" s="7" t="inlineStr">
         <is>
-          <t>KXv9 DNH2 uDd5 n165 1u</t>
+          <t>JHpXmzKUYcpbbc5cx5</t>
         </is>
       </c>
       <c r="AJ2" s="8" t="n">
@@ -3566,12 +3566,12 @@
       </c>
       <c r="AH4" s="7" t="inlineStr">
         <is>
-          <t>BBOX - 4929C743</t>
+          <t>Livebox-5B80</t>
         </is>
       </c>
       <c r="AI4" s="7" t="inlineStr">
         <is>
-          <t>KXv9 DNH2 uDd5 n165 1u</t>
+          <t>JHpXmzKUYcpbbc5cx5</t>
         </is>
       </c>
       <c r="AJ4" s="8" t="n">

</xml_diff>